<commit_message>
Estadisticos Segundo Parcial 25524
</commit_message>
<xml_diff>
--- a/Totales Generales20232.xlsx
+++ b/Totales Generales20232.xlsx
@@ -608,31 +608,31 @@
         <v>3</v>
       </c>
       <c r="E2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G2">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H2">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I2">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="J2">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="K2">
-        <v>50</v>
+        <v>74</v>
       </c>
       <c r="L2">
-        <v>142</v>
+        <v>118</v>
       </c>
       <c r="M2" s="1">
-        <v>74</v>
+        <v>61.5</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -655,13 +655,13 @@
         <v>0</v>
       </c>
       <c r="G3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H3">
         <v>6</v>
       </c>
       <c r="I3">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J3">
         <v>40</v>
@@ -702,19 +702,19 @@
         <v>8</v>
       </c>
       <c r="I4">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J4">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="K4">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="L4">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="M4" s="1">
-        <v>23.5</v>
+        <v>21.9</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -731,31 +731,31 @@
         <v>5</v>
       </c>
       <c r="E5">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F5">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G5">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="H5">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="I5">
-        <v>72</v>
+        <v>53</v>
       </c>
       <c r="J5">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="K5">
-        <v>340</v>
+        <v>367</v>
       </c>
       <c r="L5">
-        <v>259</v>
+        <v>232</v>
       </c>
       <c r="M5" s="1">
-        <v>43.2</v>
+        <v>38.7</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -933,31 +933,31 @@
         <v>10</v>
       </c>
       <c r="E10">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F10">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G10">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H10">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="I10">
-        <v>105</v>
+        <v>86</v>
       </c>
       <c r="J10">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="K10">
-        <v>505</v>
+        <v>532</v>
       </c>
       <c r="L10">
-        <v>465</v>
+        <v>438</v>
       </c>
       <c r="M10" s="1">
-        <v>47.9</v>
+        <v>45.2</v>
       </c>
     </row>
   </sheetData>
@@ -1025,34 +1025,34 @@
         <v>192</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G2">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="J2">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="K2">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="L2">
-        <v>192</v>
+        <v>174</v>
       </c>
       <c r="M2" s="1">
-        <v>100</v>
+        <v>90.59999999999999</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -1066,34 +1066,34 @@
         <v>220</v>
       </c>
       <c r="D3">
-        <v>175</v>
+        <v>2</v>
       </c>
       <c r="E3">
-        <v>45</v>
+        <v>3</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I3">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="J3">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="K3">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="L3">
-        <v>220</v>
+        <v>60</v>
       </c>
       <c r="M3" s="1">
-        <v>100</v>
+        <v>27.3</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -1110,31 +1110,31 @@
         <v>0</v>
       </c>
       <c r="E4">
-        <v>187</v>
+        <v>2</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I4">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="J4">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="K4">
-        <v>0</v>
+        <v>121</v>
       </c>
       <c r="L4">
-        <v>187</v>
+        <v>66</v>
       </c>
       <c r="M4" s="1">
-        <v>100</v>
+        <v>35.3</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -1148,34 +1148,34 @@
         <v>599</v>
       </c>
       <c r="D5">
-        <v>175</v>
+        <v>10</v>
       </c>
       <c r="E5">
-        <v>232</v>
+        <v>15</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="I5">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="J5">
-        <v>0</v>
+        <v>125</v>
       </c>
       <c r="K5">
-        <v>0</v>
+        <v>299</v>
       </c>
       <c r="L5">
-        <v>599</v>
+        <v>300</v>
       </c>
       <c r="M5" s="1">
-        <v>100</v>
+        <v>50.1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -1189,34 +1189,34 @@
         <v>128</v>
       </c>
       <c r="D6">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="E6">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G6">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H6">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="I6">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="J6">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="K6">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="L6">
-        <v>128</v>
+        <v>86</v>
       </c>
       <c r="M6" s="1">
-        <v>100</v>
+        <v>67.2</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -1230,34 +1230,34 @@
         <v>130</v>
       </c>
       <c r="D7">
-        <v>73</v>
+        <v>2</v>
       </c>
       <c r="E7">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="F7">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H7">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J7">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="K7">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="L7">
-        <v>130</v>
+        <v>46</v>
       </c>
       <c r="M7" s="1">
-        <v>100</v>
+        <v>35.4</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -1274,31 +1274,31 @@
         <v>0</v>
       </c>
       <c r="E8">
-        <v>112</v>
+        <v>2</v>
       </c>
       <c r="F8">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G8">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="H8">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I8">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="J8">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="K8">
-        <v>0</v>
+        <v>68</v>
       </c>
       <c r="L8">
-        <v>113</v>
+        <v>45</v>
       </c>
       <c r="M8" s="1">
-        <v>100</v>
+        <v>39.8</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -1312,34 +1312,34 @@
         <v>371</v>
       </c>
       <c r="D9">
-        <v>73</v>
+        <v>10</v>
       </c>
       <c r="E9">
-        <v>168</v>
+        <v>13</v>
       </c>
       <c r="F9">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="G9">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="H9">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="I9">
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="J9">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="K9">
-        <v>0</v>
+        <v>194</v>
       </c>
       <c r="L9">
-        <v>371</v>
+        <v>177</v>
       </c>
       <c r="M9" s="1">
-        <v>100</v>
+        <v>47.7</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -1350,34 +1350,34 @@
         <v>970</v>
       </c>
       <c r="D10">
-        <v>248</v>
+        <v>20</v>
       </c>
       <c r="E10">
-        <v>400</v>
+        <v>28</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="G10">
-        <v>1</v>
+        <v>38</v>
       </c>
       <c r="H10">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="I10">
-        <v>2</v>
+        <v>107</v>
       </c>
       <c r="J10">
-        <v>0</v>
+        <v>168</v>
       </c>
       <c r="K10">
-        <v>0</v>
+        <v>493</v>
       </c>
       <c r="L10">
-        <v>970</v>
+        <v>477</v>
       </c>
       <c r="M10" s="1">
-        <v>100</v>
+        <v>49.2</v>
       </c>
     </row>
   </sheetData>
@@ -1445,25 +1445,25 @@
         <v>192</v>
       </c>
       <c r="D2">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E2">
+        <v>4</v>
+      </c>
+      <c r="F2">
         <v>11</v>
       </c>
-      <c r="F2">
+      <c r="G2">
+        <v>10</v>
+      </c>
+      <c r="H2">
         <v>15</v>
       </c>
-      <c r="G2">
-        <v>14</v>
-      </c>
-      <c r="H2">
-        <v>42</v>
-      </c>
       <c r="I2">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="J2">
-        <v>52</v>
+        <v>85</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -1492,28 +1492,28 @@
         <v>3</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I3">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J3">
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="K3">
-        <v>147</v>
+        <v>160</v>
       </c>
       <c r="L3">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="M3" s="1">
-        <v>33.2</v>
+        <v>27.3</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -1539,22 +1539,22 @@
         <v>4</v>
       </c>
       <c r="H4">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I4">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J4">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="K4">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="L4">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="M4" s="1">
-        <v>23.5</v>
+        <v>19.3</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -1568,34 +1568,34 @@
         <v>599</v>
       </c>
       <c r="D5">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E5">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="F5">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G5">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="H5">
-        <v>56</v>
+        <v>28</v>
       </c>
       <c r="I5">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="J5">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="K5">
-        <v>290</v>
+        <v>311</v>
       </c>
       <c r="L5">
-        <v>309</v>
+        <v>288</v>
       </c>
       <c r="M5" s="1">
-        <v>51.6</v>
+        <v>48.1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -1609,25 +1609,25 @@
         <v>128</v>
       </c>
       <c r="D6">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E6">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F6">
+        <v>8</v>
+      </c>
+      <c r="G6">
+        <v>18</v>
+      </c>
+      <c r="H6">
         <v>13</v>
       </c>
-      <c r="G6">
-        <v>22</v>
-      </c>
-      <c r="H6">
-        <v>15</v>
-      </c>
       <c r="I6">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="J6">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="K6">
         <v>1</v>
@@ -1650,34 +1650,34 @@
         <v>130</v>
       </c>
       <c r="D7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F7">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G7">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="H7">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="I7">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J7">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="K7">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="L7">
-        <v>64</v>
+        <v>46</v>
       </c>
       <c r="M7" s="1">
-        <v>49.2</v>
+        <v>35.4</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -1694,31 +1694,31 @@
         <v>0</v>
       </c>
       <c r="E8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F8">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G8">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H8">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="I8">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J8">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="K8">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="L8">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="M8" s="1">
-        <v>38.1</v>
+        <v>38.9</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -1732,34 +1732,34 @@
         <v>371</v>
       </c>
       <c r="D9">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E9">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F9">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="G9">
+        <v>27</v>
+      </c>
+      <c r="H9">
+        <v>28</v>
+      </c>
+      <c r="I9">
         <v>33</v>
       </c>
-      <c r="H9">
-        <v>31</v>
-      </c>
-      <c r="I9">
-        <v>32</v>
-      </c>
       <c r="J9">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="K9">
-        <v>137</v>
+        <v>154</v>
       </c>
       <c r="L9">
-        <v>234</v>
+        <v>217</v>
       </c>
       <c r="M9" s="1">
-        <v>63.1</v>
+        <v>58.5</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -1773,31 +1773,31 @@
         <v>28</v>
       </c>
       <c r="E10">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="F10">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="G10">
+        <v>45</v>
+      </c>
+      <c r="H10">
         <v>56</v>
       </c>
-      <c r="H10">
-        <v>87</v>
-      </c>
       <c r="I10">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="J10">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="K10">
-        <v>427</v>
+        <v>465</v>
       </c>
       <c r="L10">
-        <v>543</v>
+        <v>505</v>
       </c>
       <c r="M10" s="1">
-        <v>56</v>
+        <v>52.1</v>
       </c>
     </row>
   </sheetData>
@@ -1859,10 +1859,10 @@
         <v>25</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E2">
         <v>3</v>
@@ -1874,7 +1874,7 @@
         <v>2</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I2">
         <v>10</v>
@@ -1897,10 +1897,10 @@
         <v>39</v>
       </c>
       <c r="C3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3">
         <v>3</v>
@@ -1909,13 +1909,13 @@
         <v>2</v>
       </c>
       <c r="G3">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H3">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I3">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J3">
         <v>0</v>
@@ -1938,22 +1938,22 @@
         <v>1</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4">
         <v>0</v>
       </c>
       <c r="F4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G4">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I4">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="J4">
         <v>0</v>
@@ -1976,19 +1976,19 @@
         <v>2</v>
       </c>
       <c r="D5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G5">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="H5">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="I5">
         <v>0</v>
@@ -2011,25 +2011,25 @@
         <v>24</v>
       </c>
       <c r="C6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E6">
         <v>1</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6">
         <v>1</v>
       </c>
       <c r="H6">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I6">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="J6">
         <v>0</v>
@@ -2049,25 +2049,25 @@
         <v>38</v>
       </c>
       <c r="C7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E7">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7">
         <v>6</v>
       </c>
-      <c r="G7">
-        <v>22</v>
-      </c>
-      <c r="H7">
-        <v>0</v>
-      </c>
       <c r="I7">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="J7">
         <v>0</v>
@@ -2093,28 +2093,28 @@
         <v>0</v>
       </c>
       <c r="E8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G8">
         <v>2</v>
       </c>
       <c r="H8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I8">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J8">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="K8">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="L8" s="1">
-        <v>51.7</v>
+        <v>44.8</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -2137,13 +2137,13 @@
         <v>0</v>
       </c>
       <c r="G9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H9">
         <v>0</v>
       </c>
       <c r="I9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J9">
         <v>37</v>
@@ -2166,31 +2166,31 @@
         <v>0</v>
       </c>
       <c r="D10">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E10">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H10">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I10">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="J10">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="K10">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="L10" s="1">
-        <v>45.7</v>
+        <v>28.6</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -2204,31 +2204,31 @@
         <v>0</v>
       </c>
       <c r="D11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E11">
         <v>0</v>
       </c>
       <c r="F11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G11">
         <v>2</v>
       </c>
       <c r="H11">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="I11">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="J11">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="K11">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="L11" s="1">
-        <v>44.4</v>
+        <v>37.8</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -2248,25 +2248,25 @@
         <v>0</v>
       </c>
       <c r="F12">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H12">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I12">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J12">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K12">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="L12" s="1">
-        <v>41.9</v>
+        <v>38.7</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -2280,31 +2280,31 @@
         <v>1</v>
       </c>
       <c r="D13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E13">
         <v>0</v>
       </c>
       <c r="F13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G13">
         <v>0</v>
       </c>
       <c r="H13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I13">
         <v>1</v>
       </c>
       <c r="J13">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="K13">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L13" s="1">
-        <v>10.5</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="14" spans="1:12">
@@ -2324,7 +2324,7 @@
         <v>1</v>
       </c>
       <c r="F14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G14">
         <v>2</v>
@@ -2333,16 +2333,16 @@
         <v>3</v>
       </c>
       <c r="I14">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J14">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K14">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="L14" s="1">
-        <v>40</v>
+        <v>36.7</v>
       </c>
     </row>
     <row r="15" spans="1:12">
@@ -2368,19 +2368,19 @@
         <v>0</v>
       </c>
       <c r="H15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I15">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J15">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="K15">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L15" s="1">
-        <v>16.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:12">
@@ -2400,25 +2400,25 @@
         <v>0</v>
       </c>
       <c r="F16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H16">
         <v>1</v>
       </c>
       <c r="I16">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J16">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="K16">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L16" s="1">
-        <v>12.5</v>
+        <v>20.8</v>
       </c>
     </row>
     <row r="17" spans="1:12">
@@ -2447,16 +2447,16 @@
         <v>0</v>
       </c>
       <c r="I17">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J17">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K17">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L17" s="1">
-        <v>6.5</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="18" spans="1:12">
@@ -2479,10 +2479,10 @@
         <v>2</v>
       </c>
       <c r="G18">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H18">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I18">
         <v>3</v>
@@ -2517,22 +2517,22 @@
         <v>0</v>
       </c>
       <c r="G19">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H19">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I19">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J19">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="K19">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L19" s="1">
-        <v>24.3</v>
+        <v>18.9</v>
       </c>
     </row>
     <row r="20" spans="1:12">
@@ -2543,25 +2543,25 @@
         <v>30</v>
       </c>
       <c r="C20">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D20">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E20">
+        <v>3</v>
+      </c>
+      <c r="F20">
         <v>5</v>
       </c>
-      <c r="F20">
+      <c r="G20">
+        <v>3</v>
+      </c>
+      <c r="H20">
+        <v>3</v>
+      </c>
+      <c r="I20">
         <v>8</v>
-      </c>
-      <c r="G20">
-        <v>2</v>
-      </c>
-      <c r="H20">
-        <v>3</v>
-      </c>
-      <c r="I20">
-        <v>5</v>
       </c>
       <c r="J20">
         <v>0</v>
@@ -2581,25 +2581,25 @@
         <v>29</v>
       </c>
       <c r="C21">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D21">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E21">
+        <v>2</v>
+      </c>
+      <c r="F21">
+        <v>4</v>
+      </c>
+      <c r="G21">
         <v>5</v>
       </c>
-      <c r="F21">
+      <c r="H21">
         <v>5</v>
       </c>
-      <c r="G21">
+      <c r="I21">
         <v>4</v>
-      </c>
-      <c r="H21">
-        <v>2</v>
-      </c>
-      <c r="I21">
-        <v>3</v>
       </c>
       <c r="J21">
         <v>0</v>
@@ -2619,25 +2619,25 @@
         <v>23</v>
       </c>
       <c r="C22">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F22">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H22">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I22">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="J22">
         <v>0</v>
@@ -2657,25 +2657,25 @@
         <v>34</v>
       </c>
       <c r="C23">
+        <v>3</v>
+      </c>
+      <c r="D23">
+        <v>3</v>
+      </c>
+      <c r="E23">
+        <v>1</v>
+      </c>
+      <c r="F23">
         <v>4</v>
       </c>
-      <c r="D23">
-        <v>3</v>
-      </c>
-      <c r="E23">
-        <v>2</v>
-      </c>
-      <c r="F23">
-        <v>5</v>
-      </c>
       <c r="G23">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H23">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I23">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="J23">
         <v>1</v>
@@ -2698,19 +2698,19 @@
         <v>1</v>
       </c>
       <c r="D24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E24">
         <v>0</v>
       </c>
       <c r="F24">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G24">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I24">
         <v>4</v>
@@ -2736,31 +2736,31 @@
         <v>0</v>
       </c>
       <c r="D25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F25">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G25">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="H25">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I25">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J25">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="K25">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="L25" s="1">
-        <v>78.3</v>
+        <v>60.9</v>
       </c>
     </row>
     <row r="26" spans="1:12">
@@ -2771,34 +2771,34 @@
         <v>31</v>
       </c>
       <c r="C26">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D26">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E26">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F26">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G26">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H26">
         <v>2</v>
       </c>
       <c r="I26">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="J26">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="K26">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="L26" s="1">
-        <v>71</v>
+        <v>51.6</v>
       </c>
     </row>
     <row r="27" spans="1:12">
@@ -2812,7 +2812,7 @@
         <v>0</v>
       </c>
       <c r="D27">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E27">
         <v>2</v>
@@ -2824,19 +2824,19 @@
         <v>2</v>
       </c>
       <c r="H27">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I27">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J27">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="K27">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="L27" s="1">
-        <v>52.4</v>
+        <v>38.1</v>
       </c>
     </row>
     <row r="28" spans="1:12">
@@ -2859,22 +2859,22 @@
         <v>0</v>
       </c>
       <c r="G28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H28">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I28">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J28">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="K28">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L28" s="1">
-        <v>16</v>
+        <v>8</v>
       </c>
     </row>
     <row r="29" spans="1:12">
@@ -2894,25 +2894,25 @@
         <v>0</v>
       </c>
       <c r="F29">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G29">
         <v>0</v>
       </c>
       <c r="H29">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I29">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="J29">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="K29">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="L29" s="1">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="30" spans="1:12">
@@ -2929,7 +2929,7 @@
         <v>0</v>
       </c>
       <c r="E30">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F30">
         <v>1</v>
@@ -2941,7 +2941,7 @@
         <v>4</v>
       </c>
       <c r="I30">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J30">
         <v>11</v>
@@ -2964,31 +2964,31 @@
         <v>0</v>
       </c>
       <c r="D31">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E31">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F31">
         <v>2</v>
       </c>
       <c r="G31">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H31">
         <v>1</v>
       </c>
       <c r="I31">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J31">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K31">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="L31" s="1">
-        <v>40.6</v>
+        <v>34.4</v>
       </c>
     </row>
     <row r="32" spans="1:12">
@@ -3011,7 +3011,7 @@
         <v>0</v>
       </c>
       <c r="G32">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H32">
         <v>1</v>
@@ -3020,13 +3020,13 @@
         <v>1</v>
       </c>
       <c r="J32">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="K32">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L32" s="1">
-        <v>20</v>
+        <v>26.7</v>
       </c>
     </row>
     <row r="33" spans="1:12">
@@ -3043,28 +3043,28 @@
         <v>0</v>
       </c>
       <c r="E33">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F33">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G33">
         <v>1</v>
       </c>
       <c r="H33">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I33">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J33">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="K33">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="L33" s="1">
-        <v>23.1</v>
+        <v>34.6</v>
       </c>
     </row>
     <row r="34" spans="1:12">
@@ -3081,28 +3081,28 @@
         <v>1</v>
       </c>
       <c r="E34">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F34">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G34">
         <v>0</v>
       </c>
       <c r="H34">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I34">
         <v>1</v>
       </c>
       <c r="J34">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K34">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L34" s="1">
-        <v>42.9</v>
+        <v>35.7</v>
       </c>
     </row>
   </sheetData>
@@ -3204,19 +3204,19 @@
         <v>31</v>
       </c>
       <c r="C4">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="E4">
         <v>0</v>
       </c>
       <c r="F4" s="1">
-        <v>38.7</v>
+        <v>41.9</v>
       </c>
       <c r="G4" s="1">
-        <v>0</v>
+        <v>58.1</v>
       </c>
       <c r="H4" s="1">
         <v>0</v>
@@ -3282,7 +3282,7 @@
         <v>38</v>
       </c>
       <c r="C7">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="D7">
         <v>0</v>
@@ -3291,7 +3291,7 @@
         <v>0</v>
       </c>
       <c r="F7" s="1">
-        <v>0</v>
+        <v>60.5</v>
       </c>
       <c r="G7" s="1">
         <v>0</v>
@@ -3311,19 +3311,19 @@
         <v>14</v>
       </c>
       <c r="D8">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="E8">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F8" s="1">
         <v>48.3</v>
       </c>
       <c r="G8" s="1">
-        <v>0</v>
+        <v>55.2</v>
       </c>
       <c r="H8" s="1">
-        <v>48.3</v>
+        <v>55.2</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -3337,7 +3337,7 @@
         <v>37</v>
       </c>
       <c r="D9">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="E9">
         <v>37</v>
@@ -3346,7 +3346,7 @@
         <v>88.09999999999999</v>
       </c>
       <c r="G9" s="1">
-        <v>0</v>
+        <v>88.09999999999999</v>
       </c>
       <c r="H9" s="1">
         <v>88.09999999999999</v>
@@ -3363,19 +3363,19 @@
         <v>19</v>
       </c>
       <c r="D10">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="E10">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="F10" s="1">
         <v>54.3</v>
       </c>
       <c r="G10" s="1">
-        <v>0</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="H10" s="1">
-        <v>54.3</v>
+        <v>71.40000000000001</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -3389,19 +3389,19 @@
         <v>25</v>
       </c>
       <c r="D11">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="E11">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F11" s="1">
         <v>55.6</v>
       </c>
       <c r="G11" s="1">
-        <v>0</v>
+        <v>62.2</v>
       </c>
       <c r="H11" s="1">
-        <v>55.6</v>
+        <v>62.2</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -3415,19 +3415,19 @@
         <v>18</v>
       </c>
       <c r="D12">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="E12">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F12" s="1">
         <v>58.1</v>
       </c>
       <c r="G12" s="1">
-        <v>0</v>
+        <v>61.3</v>
       </c>
       <c r="H12" s="1">
-        <v>58.1</v>
+        <v>61.3</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -3441,19 +3441,19 @@
         <v>34</v>
       </c>
       <c r="D13">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="E13">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F13" s="1">
         <v>89.5</v>
       </c>
       <c r="G13" s="1">
-        <v>0</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="H13" s="1">
-        <v>89.5</v>
+        <v>92.09999999999999</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -3467,19 +3467,19 @@
         <v>18</v>
       </c>
       <c r="D14">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="E14">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F14" s="1">
         <v>60</v>
       </c>
       <c r="G14" s="1">
-        <v>0</v>
+        <v>63.3</v>
       </c>
       <c r="H14" s="1">
-        <v>60</v>
+        <v>63.3</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -3490,22 +3490,22 @@
         <v>37</v>
       </c>
       <c r="C15">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D15">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="E15">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F15" s="1">
-        <v>83.8</v>
+        <v>86.5</v>
       </c>
       <c r="G15" s="1">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H15" s="1">
-        <v>83.8</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -3519,19 +3519,19 @@
         <v>21</v>
       </c>
       <c r="D16">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="E16">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F16" s="1">
         <v>87.5</v>
       </c>
       <c r="G16" s="1">
-        <v>0</v>
+        <v>79.2</v>
       </c>
       <c r="H16" s="1">
-        <v>87.5</v>
+        <v>79.2</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -3548,7 +3548,7 @@
         <v>0</v>
       </c>
       <c r="E17">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F17" s="1">
         <v>93.5</v>
@@ -3557,7 +3557,7 @@
         <v>0</v>
       </c>
       <c r="H17" s="1">
-        <v>93.5</v>
+        <v>96.8</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -3571,7 +3571,7 @@
         <v>16</v>
       </c>
       <c r="D18">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="E18">
         <v>16</v>
@@ -3580,7 +3580,7 @@
         <v>57.1</v>
       </c>
       <c r="G18" s="1">
-        <v>0</v>
+        <v>57.1</v>
       </c>
       <c r="H18" s="1">
         <v>57.1</v>
@@ -3594,22 +3594,22 @@
         <v>37</v>
       </c>
       <c r="C19">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D19">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E19">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F19" s="1">
-        <v>75.7</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="G19" s="1">
-        <v>0</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="H19" s="1">
-        <v>75.7</v>
+        <v>81.09999999999999</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -3623,7 +3623,7 @@
         <v>5</v>
       </c>
       <c r="D20">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="E20">
         <v>0</v>
@@ -3632,7 +3632,7 @@
         <v>16.7</v>
       </c>
       <c r="G20" s="1">
-        <v>0</v>
+        <v>26.7</v>
       </c>
       <c r="H20" s="1">
         <v>0</v>
@@ -3649,7 +3649,7 @@
         <v>3</v>
       </c>
       <c r="D21">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E21">
         <v>0</v>
@@ -3658,7 +3658,7 @@
         <v>10.3</v>
       </c>
       <c r="G21" s="1">
-        <v>0</v>
+        <v>13.8</v>
       </c>
       <c r="H21" s="1">
         <v>0</v>
@@ -3675,7 +3675,7 @@
         <v>8</v>
       </c>
       <c r="D22">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="E22">
         <v>0</v>
@@ -3684,7 +3684,7 @@
         <v>34.8</v>
       </c>
       <c r="G22" s="1">
-        <v>0</v>
+        <v>52.2</v>
       </c>
       <c r="H22" s="1">
         <v>0</v>
@@ -3701,7 +3701,7 @@
         <v>9</v>
       </c>
       <c r="D23">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -3710,7 +3710,7 @@
         <v>26.5</v>
       </c>
       <c r="G23" s="1">
-        <v>0</v>
+        <v>41.2</v>
       </c>
       <c r="H23" s="1">
         <v>2.9</v>
@@ -3727,7 +3727,7 @@
         <v>4</v>
       </c>
       <c r="D24">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E24">
         <v>0</v>
@@ -3736,7 +3736,7 @@
         <v>33.3</v>
       </c>
       <c r="G24" s="1">
-        <v>0</v>
+        <v>33.3</v>
       </c>
       <c r="H24" s="1">
         <v>0</v>
@@ -3753,19 +3753,19 @@
         <v>5</v>
       </c>
       <c r="D25">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="E25">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="F25" s="1">
         <v>21.7</v>
       </c>
       <c r="G25" s="1">
-        <v>0</v>
+        <v>39.1</v>
       </c>
       <c r="H25" s="1">
-        <v>21.7</v>
+        <v>39.1</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -3779,19 +3779,19 @@
         <v>9</v>
       </c>
       <c r="D26">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="E26">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="F26" s="1">
         <v>29</v>
       </c>
       <c r="G26" s="1">
-        <v>0</v>
+        <v>48.4</v>
       </c>
       <c r="H26" s="1">
-        <v>29</v>
+        <v>48.4</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -3805,19 +3805,19 @@
         <v>10</v>
       </c>
       <c r="D27">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="E27">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F27" s="1">
         <v>47.6</v>
       </c>
       <c r="G27" s="1">
-        <v>0</v>
+        <v>61.9</v>
       </c>
       <c r="H27" s="1">
-        <v>47.6</v>
+        <v>61.9</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -3831,19 +3831,19 @@
         <v>21</v>
       </c>
       <c r="D28">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="E28">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F28" s="1">
         <v>84</v>
       </c>
       <c r="G28" s="1">
-        <v>0</v>
+        <v>92</v>
       </c>
       <c r="H28" s="1">
-        <v>84</v>
+        <v>92</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -3857,19 +3857,19 @@
         <v>21</v>
       </c>
       <c r="D29">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="E29">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F29" s="1">
         <v>70</v>
       </c>
       <c r="G29" s="1">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="H29" s="1">
-        <v>70</v>
+        <v>80</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -3883,7 +3883,7 @@
         <v>11</v>
       </c>
       <c r="D30">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="E30">
         <v>11</v>
@@ -3892,7 +3892,7 @@
         <v>42.3</v>
       </c>
       <c r="G30" s="1">
-        <v>0</v>
+        <v>42.3</v>
       </c>
       <c r="H30" s="1">
         <v>42.3</v>
@@ -3909,19 +3909,19 @@
         <v>19</v>
       </c>
       <c r="D31">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="E31">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F31" s="1">
         <v>59.4</v>
       </c>
       <c r="G31" s="1">
-        <v>0</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="H31" s="1">
-        <v>59.4</v>
+        <v>65.59999999999999</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -3935,19 +3935,19 @@
         <v>12</v>
       </c>
       <c r="D32">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="E32">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F32" s="1">
         <v>80</v>
       </c>
       <c r="G32" s="1">
-        <v>0</v>
+        <v>73.3</v>
       </c>
       <c r="H32" s="1">
-        <v>80</v>
+        <v>73.3</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -3961,19 +3961,19 @@
         <v>20</v>
       </c>
       <c r="D33">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="E33">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F33" s="1">
         <v>76.90000000000001</v>
       </c>
       <c r="G33" s="1">
-        <v>0</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="H33" s="1">
-        <v>76.90000000000001</v>
+        <v>65.40000000000001</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -3987,19 +3987,19 @@
         <v>8</v>
       </c>
       <c r="D34">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="E34">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F34" s="1">
         <v>57.1</v>
       </c>
       <c r="G34" s="1">
-        <v>0</v>
+        <v>57.1</v>
       </c>
       <c r="H34" s="1">
-        <v>57.1</v>
+        <v>64.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>